<commit_message>
upload exce dan import excel
</commit_message>
<xml_diff>
--- a/docs/Dokumen_Testing_POS.xlsx
+++ b/docs/Dokumen_Testing_POS.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4393C7C9-49DA-405F-A7C9-082D32B48FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032A6B41-4582-4003-B580-8B77DCAC5697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="867" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="867" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daftar Isi" sheetId="1" r:id="rId1"/>
@@ -49,12 +49,23 @@
     <sheet name="Dummy - Pengeluaran" sheetId="39" r:id="rId39"/>
     <sheet name="Dummy - Transaksi" sheetId="40" r:id="rId40"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2290" uniqueCount="1159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2270" uniqueCount="1145">
   <si>
     <t>DOKUMEN TESTING APLIKASI POS</t>
   </si>
@@ -2895,9 +2906,6 @@
     <t>min_stock</t>
   </si>
   <si>
-    <t>8991002100016</t>
-  </si>
-  <si>
     <t>SKU-0001</t>
   </si>
   <si>
@@ -2913,27 +2921,15 @@
     <t>200</t>
   </si>
   <si>
-    <t>8992388123456</t>
-  </si>
-  <si>
     <t>SKU-0002</t>
   </si>
   <si>
     <t>Teh Botol Sosro 450ml</t>
   </si>
   <si>
-    <t>4000</t>
-  </si>
-  <si>
-    <t>5000</t>
-  </si>
-  <si>
     <t>150</t>
   </si>
   <si>
-    <t>8996001600028</t>
-  </si>
-  <si>
     <t>SKU-0003</t>
   </si>
   <si>
@@ -2970,54 +2966,33 @@
     <t>50</t>
   </si>
   <si>
-    <t>8991234567890</t>
-  </si>
-  <si>
     <t>SKU-0005</t>
   </si>
   <si>
     <t>Sampoerna A Mild 16</t>
   </si>
   <si>
-    <t>22000</t>
-  </si>
-  <si>
-    <t>24000</t>
-  </si>
-  <si>
     <t>80</t>
   </si>
   <si>
-    <t>8990001112223</t>
-  </si>
-  <si>
     <t>SKU-0006</t>
   </si>
   <si>
     <t>Chitato Sapi Panggang 68g</t>
   </si>
   <si>
-    <t>8500</t>
-  </si>
-  <si>
     <t>10000</t>
   </si>
   <si>
     <t>true - stok di bawah min_stock (untuk uji notifikasi stok)</t>
   </si>
   <si>
-    <t>8990004445556</t>
-  </si>
-  <si>
     <t>SKU-0007</t>
   </si>
   <si>
     <t>Kopi Kapal Api Sachet</t>
   </si>
   <si>
-    <t>1200</t>
-  </si>
-  <si>
     <t>1500</t>
   </si>
   <si>
@@ -3073,12 +3048,6 @@
   </si>
   <si>
     <t>Dus (isi 24)</t>
-  </si>
-  <si>
-    <t>78000</t>
-  </si>
-  <si>
-    <t>65000</t>
   </si>
   <si>
     <t>DUMMY DATA - DATA HARGA GROSIR (TIER PRICE) - lanjutan sheet Produk</t>
@@ -7150,7 +7119,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7176,7 +7145,7 @@
         <v>5</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7202,7 +7171,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7228,7 +7197,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7254,7 +7223,7 @@
         <v>5</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7280,7 +7249,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7306,7 +7275,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -7332,7 +7301,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -7384,7 +7353,7 @@
         <v>5</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -9943,14 +9912,14 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="2">
+        <v>8991002100016</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>900</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>901</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>902</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>864</v>
@@ -9958,14 +9927,14 @@
       <c r="E4" s="2" t="s">
         <v>879</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>903</v>
-      </c>
-      <c r="G4" s="2" t="s">
+      <c r="F4" s="2">
+        <v>2500</v>
+      </c>
+      <c r="G4" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>904</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>905</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>63</v>
@@ -9975,14 +9944,14 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="2">
+        <v>8992388123456</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>905</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>906</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>907</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>908</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>867</v>
@@ -9990,14 +9959,14 @@
       <c r="E5" s="2" t="s">
         <v>879</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>909</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>910</v>
+      <c r="F5" s="2">
+        <v>4000</v>
+      </c>
+      <c r="G5" s="2">
+        <v>5000</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>48</v>
@@ -10007,14 +9976,14 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>912</v>
+      <c r="A6" s="2">
+        <v>8996001600028</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>867</v>
@@ -10022,17 +9991,17 @@
       <c r="E6" s="2" t="s">
         <v>879</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>915</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>916</v>
+      <c r="F6" s="2">
+        <v>2800</v>
+      </c>
+      <c r="G6" s="2">
+        <v>3500</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>850</v>
@@ -10040,13 +10009,13 @@
     </row>
     <row r="7" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>870</v>
@@ -10055,13 +10024,13 @@
         <v>879</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>18</v>
@@ -10071,14 +10040,14 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>925</v>
+      <c r="A8" s="2">
+        <v>8991234567890</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>926</v>
+        <v>920</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>927</v>
+        <v>921</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>873</v>
@@ -10086,14 +10055,14 @@
       <c r="E8" s="2" t="s">
         <v>879</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>928</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>929</v>
+      <c r="F8" s="2">
+        <v>22000</v>
+      </c>
+      <c r="G8" s="2">
+        <v>24000</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>930</v>
+        <v>922</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>33</v>
@@ -10103,14 +10072,14 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>931</v>
+      <c r="A9" s="2">
+        <v>8990001112223</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>932</v>
+        <v>923</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>933</v>
+        <v>924</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>864</v>
@@ -10118,11 +10087,11 @@
       <c r="E9" s="2" t="s">
         <v>879</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>934</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>935</v>
+      <c r="F9" s="2">
+        <v>8500</v>
+      </c>
+      <c r="G9" s="2">
+        <v>10000</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>18</v>
@@ -10131,18 +10100,18 @@
         <v>33</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>936</v>
+        <v>926</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>937</v>
+      <c r="A10" s="2">
+        <v>8990004445556</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>938</v>
+        <v>927</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>939</v>
+        <v>928</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>867</v>
@@ -10150,31 +10119,31 @@
       <c r="E10" s="2" t="s">
         <v>879</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>940</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>941</v>
+      <c r="F10" s="2">
+        <v>1200</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1500</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>63</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>943</v>
+        <v>931</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>944</v>
+        <v>932</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>945</v>
+        <v>933</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>946</v>
+        <v>934</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>864</v>
@@ -10183,10 +10152,10 @@
         <v>879</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>947</v>
+        <v>935</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>941</v>
+        <v>929</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>33</v>
@@ -10195,7 +10164,7 @@
         <v>18</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>948</v>
+        <v>936</v>
       </c>
     </row>
   </sheetData>
@@ -10221,7 +10190,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>949</v>
+        <v>937</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -10232,16 +10201,16 @@
     </row>
     <row r="3" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>950</v>
+        <v>938</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>951</v>
+        <v>939</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>895</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>952</v>
+        <v>940</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>897</v>
@@ -10250,15 +10219,15 @@
         <v>896</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>953</v>
+        <v>941</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>954</v>
+        <v>942</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>879</v>
@@ -10267,10 +10236,10 @@
         <v>6</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>850</v>
@@ -10278,22 +10247,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>955</v>
+        <v>943</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>883</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>956</v>
+        <v>944</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>957</v>
+        <v>945</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>958</v>
+        <v>946</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>854</v>
@@ -10301,10 +10270,10 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>954</v>
+        <v>942</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>879</v>
@@ -10313,10 +10282,10 @@
         <v>6</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>850</v>
@@ -10324,10 +10293,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>959</v>
+        <v>947</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>883</v>
@@ -10335,11 +10304,11 @@
       <c r="D7" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>960</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>961</v>
+      <c r="E7" s="2">
+        <v>78000</v>
+      </c>
+      <c r="F7" s="2">
+        <v>65000</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>854</v>
@@ -10365,7 +10334,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>962</v>
+        <v>948</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -10373,58 +10342,58 @@
     </row>
     <row r="3" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>938</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>949</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>950</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>963</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>964</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>965</v>
+        <v>951</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>966</v>
+        <v>952</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>39</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>967</v>
+        <v>953</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>956</v>
+        <v>944</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>968</v>
+        <v>954</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>969</v>
+        <v>955</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>970</v>
+        <v>956</v>
       </c>
     </row>
   </sheetData>
@@ -10452,7 +10421,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>971</v>
+        <v>957</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -10463,22 +10432,22 @@
     </row>
     <row r="3" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>972</v>
+        <v>958</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>860</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>973</v>
+        <v>959</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>974</v>
+        <v>960</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>975</v>
+        <v>961</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>976</v>
+        <v>962</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>848</v>
@@ -10486,22 +10455,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>977</v>
+        <v>963</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>978</v>
+        <v>964</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>979</v>
+        <v>965</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>980</v>
+        <v>966</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>981</v>
+        <v>967</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>982</v>
+        <v>968</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>850</v>
@@ -10509,22 +10478,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>983</v>
+        <v>969</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>984</v>
+        <v>970</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>985</v>
+        <v>971</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>986</v>
+        <v>972</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>987</v>
+        <v>973</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>988</v>
+        <v>974</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>850</v>
@@ -10532,22 +10501,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>989</v>
+        <v>975</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>990</v>
+        <v>976</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>991</v>
+        <v>977</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>992</v>
+        <v>978</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>993</v>
+        <v>979</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>994</v>
+        <v>980</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>850</v>
@@ -10555,22 +10524,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>995</v>
+        <v>981</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>996</v>
+        <v>982</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>997</v>
+        <v>983</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>998</v>
+        <v>984</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>999</v>
+        <v>985</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>1000</v>
+        <v>986</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>854</v>
@@ -10599,7 +10568,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>1001</v>
+        <v>987</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -10611,106 +10580,106 @@
     </row>
     <row r="3" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>1002</v>
+        <v>988</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1003</v>
+        <v>989</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1004</v>
+        <v>990</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>1005</v>
+        <v>991</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1006</v>
+        <v>992</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>1007</v>
+        <v>993</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>1008</v>
+        <v>994</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>1009</v>
+        <v>995</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>1010</v>
+        <v>996</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>978</v>
+        <v>964</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1011</v>
+        <v>997</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1012</v>
+        <v>998</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>935</v>
+        <v>925</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1013</v>
+        <v>999</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>1014</v>
+        <v>1000</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>1013</v>
+        <v>999</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>1015</v>
+        <v>1001</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>984</v>
+        <v>970</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1016</v>
+        <v>1002</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1017</v>
+        <v>1003</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1018</v>
+        <v>1004</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>1019</v>
+        <v>1005</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>1020</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>1021</v>
+        <v>1007</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>990</v>
+        <v>976</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1022</v>
+        <v>1008</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1023</v>
+        <v>1009</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1024</v>
+        <v>1010</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>1025</v>
+        <v>1011</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1026</v>
+        <v>1012</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
     </row>
   </sheetData>
@@ -10737,7 +10706,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>1027</v>
+        <v>1013</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -10747,19 +10716,19 @@
     </row>
     <row r="3" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>1028</v>
+        <v>1014</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>860</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>974</v>
+        <v>960</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>973</v>
+        <v>959</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1029</v>
+        <v>1015</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>848</v>
@@ -10767,19 +10736,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>1030</v>
+        <v>1016</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1031</v>
+        <v>1017</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1032</v>
+        <v>1018</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1033</v>
+        <v>1019</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1034</v>
+        <v>1020</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>850</v>
@@ -10787,19 +10756,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>1035</v>
+        <v>1021</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1036</v>
+        <v>1022</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1037</v>
+        <v>1023</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1038</v>
+        <v>1024</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1039</v>
+        <v>1025</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>850</v>
@@ -10807,19 +10776,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>1040</v>
+        <v>1026</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1041</v>
+        <v>1027</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1042</v>
+        <v>1028</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1043</v>
+        <v>1029</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1044</v>
+        <v>1030</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>850</v>
@@ -10827,19 +10796,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>1045</v>
+        <v>1031</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1046</v>
+        <v>1032</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1047</v>
+        <v>1033</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1048</v>
+        <v>1034</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>854</v>
@@ -10869,7 +10838,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>1049</v>
+        <v>1035</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -10880,94 +10849,94 @@
     </row>
     <row r="3" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>1050</v>
+        <v>1036</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1051</v>
+        <v>1037</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1007</v>
+        <v>993</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>1009</v>
+        <v>995</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1052</v>
+        <v>1038</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>1053</v>
+        <v>1039</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>1054</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>1031</v>
+        <v>1017</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1055</v>
+        <v>1041</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1056</v>
+        <v>1042</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1056</v>
+        <v>1042</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1026</v>
+        <v>1012</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>1057</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>1036</v>
+        <v>1022</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1058</v>
+        <v>1044</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1034</v>
+        <v>1020</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1059</v>
+        <v>1045</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1059</v>
+        <v>1045</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1019</v>
+        <v>1005</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>1060</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>1041</v>
+        <v>1027</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1061</v>
+        <v>1047</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1062</v>
+        <v>1048</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1062</v>
+        <v>1048</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>1014</v>
+        <v>1000</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1063</v>
+        <v>1049</v>
       </c>
     </row>
   </sheetData>
@@ -10991,7 +10960,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>1064</v>
+        <v>1050</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -11002,10 +10971,10 @@
         <v>860</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1065</v>
+        <v>1051</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1066</v>
+        <v>1052</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>848</v>
@@ -11013,13 +10982,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>1067</v>
+        <v>1053</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1068</v>
+        <v>1054</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1069</v>
+        <v>1055</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>850</v>
@@ -11027,13 +10996,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>1070</v>
+        <v>1056</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1069</v>
+        <v>1055</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1071</v>
+        <v>1057</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>850</v>
@@ -11041,13 +11010,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>1072</v>
+        <v>1058</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1071</v>
+        <v>1057</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1068</v>
+        <v>1054</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>850</v>
@@ -11077,7 +11046,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>1073</v>
+        <v>1059</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -11092,25 +11061,25 @@
         <v>852</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1074</v>
+        <v>1060</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1075</v>
+        <v>1061</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>1076</v>
+        <v>1062</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1077</v>
+        <v>1063</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>1078</v>
+        <v>1064</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>1053</v>
+        <v>1039</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>1079</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -11118,25 +11087,25 @@
         <v>826</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>930</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>1067</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>1034</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>1080</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>1080</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>942</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>1081</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>1082</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -11144,25 +11113,25 @@
         <v>830</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>1070</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>1083</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>1084</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>1039</v>
+        <v>1025</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1085</v>
+        <v>1071</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>1081</v>
+        <v>1067</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>1086</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -11170,10 +11139,10 @@
         <v>826</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1072</v>
+        <v>1058</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1087</v>
+        <v>1073</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>5</v>
@@ -11185,10 +11154,10 @@
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1088</v>
+        <v>1074</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>1089</v>
+        <v>1075</v>
       </c>
     </row>
   </sheetData>
@@ -11215,7 +11184,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>1090</v>
+        <v>1076</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -11225,7 +11194,7 @@
     </row>
     <row r="3" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>1091</v>
+        <v>1077</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>894</v>
@@ -11234,30 +11203,30 @@
         <v>862</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>1092</v>
+        <v>1078</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1093</v>
+        <v>1079</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>1094</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>1022</v>
+        <v>1008</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1095</v>
+        <v>1081</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1096</v>
+        <v>1082</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1097</v>
+        <v>1083</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1098</v>
+        <v>1084</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>826</v>
@@ -11265,19 +11234,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>1022</v>
+        <v>1008</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1099</v>
+        <v>1085</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1100</v>
+        <v>1086</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1101</v>
+        <v>1087</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1102</v>
+        <v>1088</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>822</v>
@@ -11285,19 +11254,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>1103</v>
+        <v>1089</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1104</v>
+        <v>1090</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1105</v>
+        <v>1091</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1106</v>
+        <v>1092</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1098</v>
+        <v>1084</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>830</v>
@@ -11305,19 +11274,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>1103</v>
+        <v>1089</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1107</v>
+        <v>1093</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1108</v>
+        <v>1094</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1109</v>
+        <v>1095</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1098</v>
+        <v>1084</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>817</v>
@@ -11408,7 +11377,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -11434,7 +11403,7 @@
         <v>5</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -11460,7 +11429,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -11486,7 +11455,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -11512,7 +11481,7 @@
         <v>5</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -11538,7 +11507,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -11564,7 +11533,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -11590,7 +11559,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -11616,7 +11585,7 @@
         <v>5</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -11636,13 +11605,13 @@
         <v>227</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>1140</v>
+        <v>1126</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>5</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -11653,19 +11622,19 @@
         <v>119</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1136</v>
+        <v>1122</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1137</v>
+        <v>1123</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>1138</v>
+        <v>1124</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>1139</v>
+        <v>1125</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
   </sheetData>
@@ -11693,7 +11662,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>1110</v>
+        <v>1096</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -11707,54 +11676,54 @@
     </row>
     <row r="3" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>1111</v>
+        <v>1097</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>852</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1005</v>
+        <v>991</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>1093</v>
+        <v>1079</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1112</v>
+        <v>1098</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>1007</v>
+        <v>993</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>1050</v>
+        <v>1036</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>1113</v>
+        <v>1099</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>1053</v>
+        <v>1039</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>1114</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>1115</v>
+        <v>1101</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>826</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1116</v>
+        <v>1102</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1098</v>
+        <v>1084</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>935</v>
+        <v>925</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1117</v>
+        <v>1103</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>159</v>
@@ -11763,30 +11732,30 @@
         <v>854</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>1118</v>
+        <v>1104</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>1119</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>1120</v>
+        <v>1106</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>826</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1121</v>
+        <v>1107</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1122</v>
+        <v>1108</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1123</v>
+        <v>1109</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1123</v>
+        <v>1109</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>159</v>
@@ -11795,30 +11764,30 @@
         <v>854</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>1118</v>
+        <v>1104</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>1124</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>1125</v>
+        <v>1111</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>830</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1126</v>
+        <v>1112</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1102</v>
+        <v>1088</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>159</v>
@@ -11827,62 +11796,62 @@
         <v>854</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>1118</v>
+        <v>1104</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>1127</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>1055</v>
+        <v>1041</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>826</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1128</v>
+        <v>1114</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1129</v>
+        <v>1115</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>942</v>
+        <v>930</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>1056</v>
+        <v>1042</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>1031</v>
+        <v>1017</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>850</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>1118</v>
+        <v>1104</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>1119</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>1061</v>
+        <v>1047</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>830</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1130</v>
+        <v>1116</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1098</v>
+        <v>1084</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>957</v>
+        <v>945</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>957</v>
+        <v>945</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>159</v>
@@ -11891,30 +11860,30 @@
         <v>854</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>1118</v>
+        <v>1104</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>1119</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>1131</v>
+        <v>1117</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>826</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1132</v>
+        <v>1118</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1098</v>
+        <v>1084</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>1133</v>
+        <v>1119</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>1133</v>
+        <v>1119</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>159</v>
@@ -11923,10 +11892,10 @@
         <v>854</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>1134</v>
+        <v>1120</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>1119</v>
+        <v>1105</v>
       </c>
     </row>
   </sheetData>
@@ -12502,7 +12471,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -12528,7 +12497,7 @@
         <v>5</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -12539,7 +12508,7 @@
         <v>229</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1144</v>
+        <v>1130</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>317</v>
@@ -12554,7 +12523,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -12580,7 +12549,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -12606,7 +12575,7 @@
         <v>5</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -12632,7 +12601,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -12658,7 +12627,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -12684,7 +12653,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -12695,22 +12664,22 @@
         <v>119</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1149</v>
+        <v>1135</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1150</v>
+        <v>1136</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>299</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>1151</v>
+        <v>1137</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>5</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
   </sheetData>
@@ -12798,7 +12767,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -12824,7 +12793,7 @@
         <v>5</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -12850,7 +12819,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -12861,13 +12830,13 @@
         <v>229</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1141</v>
+        <v>1127</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1142</v>
+        <v>1128</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1143</v>
+        <v>1129</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>292</v>
@@ -12876,7 +12845,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -12902,7 +12871,7 @@
         <v>5</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -12913,13 +12882,13 @@
         <v>229</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1145</v>
+        <v>1131</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>1146</v>
+        <v>1132</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>1147</v>
+        <v>1133</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>300</v>
@@ -12928,7 +12897,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -12954,7 +12923,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -12965,7 +12934,7 @@
         <v>128</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>1148</v>
+        <v>1134</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>306</v>
@@ -12980,7 +12949,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -12991,22 +12960,22 @@
         <v>119</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1152</v>
+        <v>1138</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1153</v>
+        <v>1139</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>1158</v>
+        <v>1144</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>1154</v>
+        <v>1140</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>5</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
   </sheetData>
@@ -13094,7 +13063,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
@@ -13120,7 +13089,7 @@
         <v>5</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13146,7 +13115,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13172,7 +13141,7 @@
         <v>5</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13198,7 +13167,7 @@
         <v>5</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13224,7 +13193,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -13250,7 +13219,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13276,7 +13245,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13302,7 +13271,7 @@
         <v>5</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -13327,8 +13296,8 @@
       <c r="G13" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>5</v>
+      <c r="H13" s="3" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13353,8 +13322,8 @@
       <c r="G14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>5</v>
+      <c r="H14" s="3" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13379,8 +13348,8 @@
       <c r="G15" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>5</v>
+      <c r="H15" s="3" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
@@ -13405,8 +13374,8 @@
       <c r="G16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>5</v>
+      <c r="H16" s="3" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -13431,8 +13400,8 @@
       <c r="G17" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>5</v>
+      <c r="H17" s="3" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
@@ -13457,8 +13426,8 @@
       <c r="G18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>5</v>
+      <c r="H18" s="3" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -13509,34 +13478,34 @@
       <c r="G20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>5</v>
+      <c r="H20" s="3" t="s">
+        <v>1121</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>119</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>1155</v>
+        <v>1141</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>1156</v>
+        <v>1142</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>387</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>1157</v>
+        <v>1143</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>5</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>1135</v>
+        <v>1121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>